<commit_message>
ajout Simon et Mr. X
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/techinfo/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA6E249-5DA8-C141-B1C2-481C16763334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D147A097-15A3-9F40-8115-C0A8202C1448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="16960" windowHeight="17780" xr2:uid="{6B795B45-6C14-B04F-B93D-A59A5BE3A68D}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="92">
   <si>
     <t>Lundi</t>
   </si>
@@ -295,6 +295,24 @@
   </si>
   <si>
     <t>Dévelopment Web 2</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>Analyse de données en gestion</t>
+  </si>
+  <si>
+    <t>Fonctionnement de l'ordinateur</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Nano-ordinateurs</t>
+  </si>
+  <si>
+    <t>B121</t>
   </si>
 </sst>
 </file>
@@ -351,7 +369,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -380,8 +398,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29040E5A-5519-964C-B6DE-2A568682510C}" name="Table1" displayName="Table1" ref="A1:I38" totalsRowShown="0">
-  <autoFilter ref="A1:I38" xr:uid="{29040E5A-5519-964C-B6DE-2A568682510C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29040E5A-5519-964C-B6DE-2A568682510C}" name="Table1" displayName="Table1" ref="A1:I49" totalsRowShown="0">
+  <autoFilter ref="A1:I49" xr:uid="{29040E5A-5519-964C-B6DE-2A568682510C}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I23">
     <sortCondition ref="E2:E23"/>
     <sortCondition ref="A2:A23"/>
@@ -718,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46DF1DC5-63E0-A14F-8B6A-86AB73F394B2}">
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1165,10 +1183,10 @@
       <c r="A16" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D16" s="2">
@@ -1194,10 +1212,10 @@
       <c r="A17" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D17" s="2">
@@ -1426,10 +1444,10 @@
       <c r="A25" t="s">
         <v>0</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D25" s="2">
@@ -1484,10 +1502,10 @@
       <c r="A27" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D27" s="2">
@@ -1513,10 +1531,10 @@
       <c r="A28" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D28" s="2">
@@ -1542,10 +1560,10 @@
       <c r="A29" t="s">
         <v>20</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D29" s="2">
@@ -1600,10 +1618,10 @@
       <c r="A31" t="s">
         <v>0</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D31" s="2">
@@ -1629,10 +1647,10 @@
       <c r="A32" t="s">
         <v>0</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D32" s="2">
@@ -1687,10 +1705,10 @@
       <c r="A34" t="s">
         <v>19</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D34" s="2">
@@ -1774,10 +1792,10 @@
       <c r="A37" t="s">
         <v>20</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D37" s="2">
@@ -1803,10 +1821,10 @@
       <c r="A38" t="s">
         <v>20</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D38" s="2">
@@ -1826,6 +1844,325 @@
       </c>
       <c r="I38">
         <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D39" s="2">
+        <v>2</v>
+      </c>
+      <c r="E39" t="s">
+        <v>27</v>
+      </c>
+      <c r="F39" t="s">
+        <v>87</v>
+      </c>
+      <c r="G39" t="s">
+        <v>21</v>
+      </c>
+      <c r="H39" t="s">
+        <v>86</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D40" s="2">
+        <v>2</v>
+      </c>
+      <c r="E40" t="s">
+        <v>27</v>
+      </c>
+      <c r="F40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G40" t="s">
+        <v>21</v>
+      </c>
+      <c r="H40" t="s">
+        <v>86</v>
+      </c>
+      <c r="I40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>19</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D41" s="2">
+        <v>2</v>
+      </c>
+      <c r="E41" t="s">
+        <v>27</v>
+      </c>
+      <c r="F41" t="s">
+        <v>88</v>
+      </c>
+      <c r="G41" t="s">
+        <v>2</v>
+      </c>
+      <c r="H41" t="s">
+        <v>86</v>
+      </c>
+      <c r="I41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>19</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D42" s="2">
+        <v>2</v>
+      </c>
+      <c r="E42" t="s">
+        <v>27</v>
+      </c>
+      <c r="F42" t="s">
+        <v>88</v>
+      </c>
+      <c r="G42" t="s">
+        <v>2</v>
+      </c>
+      <c r="H42" t="s">
+        <v>86</v>
+      </c>
+      <c r="I42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D43" s="2">
+        <v>2</v>
+      </c>
+      <c r="E43" t="s">
+        <v>27</v>
+      </c>
+      <c r="F43" t="s">
+        <v>88</v>
+      </c>
+      <c r="G43" t="s">
+        <v>2</v>
+      </c>
+      <c r="H43" t="s">
+        <v>86</v>
+      </c>
+      <c r="I43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D44" s="2">
+        <v>2</v>
+      </c>
+      <c r="E44" t="s">
+        <v>27</v>
+      </c>
+      <c r="F44" t="s">
+        <v>88</v>
+      </c>
+      <c r="G44" t="s">
+        <v>2</v>
+      </c>
+      <c r="H44" t="s">
+        <v>86</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>5</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D45" s="2">
+        <v>2</v>
+      </c>
+      <c r="E45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F45" t="s">
+        <v>87</v>
+      </c>
+      <c r="G45" t="s">
+        <v>21</v>
+      </c>
+      <c r="H45" t="s">
+        <v>86</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>5</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D46" s="2">
+        <v>2</v>
+      </c>
+      <c r="E46" t="s">
+        <v>27</v>
+      </c>
+      <c r="F46" t="s">
+        <v>87</v>
+      </c>
+      <c r="G46" t="s">
+        <v>2</v>
+      </c>
+      <c r="H46" t="s">
+        <v>86</v>
+      </c>
+      <c r="I46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>0</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D47" s="2">
+        <v>2</v>
+      </c>
+      <c r="E47" t="s">
+        <v>89</v>
+      </c>
+      <c r="F47" t="s">
+        <v>87</v>
+      </c>
+      <c r="G47" t="s">
+        <v>91</v>
+      </c>
+      <c r="H47" t="s">
+        <v>89</v>
+      </c>
+      <c r="I47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>0</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D48" s="2">
+        <v>3</v>
+      </c>
+      <c r="E48" t="s">
+        <v>89</v>
+      </c>
+      <c r="F48" t="s">
+        <v>90</v>
+      </c>
+      <c r="G48" t="s">
+        <v>2</v>
+      </c>
+      <c r="H48" t="s">
+        <v>89</v>
+      </c>
+      <c r="I48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>19</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D49" s="2">
+        <v>2</v>
+      </c>
+      <c r="E49" t="s">
+        <v>89</v>
+      </c>
+      <c r="F49" t="s">
+        <v>87</v>
+      </c>
+      <c r="G49" t="s">
+        <v>21</v>
+      </c>
+      <c r="H49" t="s">
+        <v>89</v>
+      </c>
+      <c r="I49">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>